<commit_message>
docs(state): close monorepo bootstrap [R-001]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbbe609a94fe6405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Rd9ffae5f9e08499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R5281c784f09c4ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Ra88293b40c3647bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R486f71848f1d4fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R8e0656c55bf34d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Red754b3f4e034903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R99b1a9c2e2584d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R03a020807e4c4926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R82cadf81c1fe46c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R1bb771829ec04e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rcea8f5695dda49d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Re49b14150b8b4fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R74900d517ef64b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R7a333a2784b7412a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="Rbf30424629834973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R56f9982514ec4c2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R52ab312bf27f43ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rfe9c7bbfcb3e4cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R4ae80a3db4ac48e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rd6336210097e425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Ra8ef5ec2e43646e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R9bbdac122ee443a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R23d983b4e0b54559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R87e16378cec04e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Rcdd268ce4c2e44a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="Rfe5d0e44ed5744c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R3f6c0464f8ca4e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R1e3dd2b250ac45c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R821ecf18f1d84721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Re9aa046ae6e144a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Raa88f68917964720"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R5e9b3d1fed294da5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Re06998f4bed2431b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R1c322b1a273146f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R9c5895f5b71d407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R2c199b36166f4ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R1ed7fc4d538c4bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Redeac162ebee46b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="Rd5683193bee24f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R47221c194dbc4565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R56e91dae03db40cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R6b712a79253b4aa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R16da6693456342a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R839f10c154824757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R21e1a3d00c3b4fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R9451357a51134cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R859e328057004a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R80f0cdbfee934eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R0a82bb8127134445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Ra4f2147d959741cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R4bd1322932774738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rc16da02fedbd474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Rb1bb4276559242ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Raf0bfe3f87b64467"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R7166dd472ac14dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Re5f45c15dbd24c74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R5c39db710e6c4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R2d2d44852a834fb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R594b761480e547bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rccaa6c3739ab4d79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R3da6f002791b4da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R53434dee85974d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R811d5e952e86496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R1137bd330331448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R24fe666cb85f4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R25283bf47a754fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rc91414faee36438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Re9ff0c04f09641c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Rc27ed19f114f430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Re129f1cbb9904d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rbe55f94bbad54bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R5499cef0e3f34d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rdd1f17b2cb30447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R923b51ac0595453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Rf62e835aadc647d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rdf48a97b2ae148b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R7c58b57d949a4ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rd12114bcffd94601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rf6eb86bd258d4596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rb8ca52395bd34c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R42dc08fe01ad4ad8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R2f791a86bea747a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R25f6899593e44230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R2627ba994766437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R8209352158df40a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R8dd65bdd0cd84139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Raf1c3ff93da0451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R0f40aef933c14f11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R90feb16396af48c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R551da609cef746cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R0fcc51ad90a5453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rf7245d1c83844a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rd1e09b7f635e48ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R6171d3d61e864a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R9530e900431c407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R8445655acc534906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R0c7d5c727fc641b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Raa5c2c4fa6674e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R230e483b87e74047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R1ff023cfe0924178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R13ebd64926b84e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R52389870c8024969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rffee81e084c34d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R19773a28afd04520"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R2862f88e3dc34d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R5aa81de6bf5a4f5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R5693377c424a467f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R5f6c0f75bb9e4c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rafb0645ceffe4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rfc5b57c03fe240bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R9aeb6de9abdc4eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R0af15f49ea724801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rb938ba0233104cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rb2932757ae824c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R2c590a6204d44fe0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Raae9fa6d54984c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R19798d42e55b4536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R0c8b60a5550749d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rd0431f8af02b4055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R7f4f575efdca4c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rff01e373444f4e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rf404238e04de469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R7dfd9445dc784c39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2310,9 +2310,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -2381,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R746a0e22665c455e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33dc2c58b3e24603"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2704,15 +2702,15 @@
       </x:c>
       <x:c r="B5" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$B$4:$B$222,"MVP")</x:f>
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0</x:v>
+        <x:v>0.009433962264150943</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2805,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F8)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3974,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re77cd311e3024246"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra941cc7dbd444fa7"/>
 </x:worksheet>
 </file>
 
@@ -10687,19 +10685,46 @@
       <x:c r="M11" s="32" t="n"/>
     </x:row>
     <x:row r="12" s="40" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A12" s="32" t="n"/>
-      <x:c r="B12" s="32" t="n"/>
-      <x:c r="C12" s="32" t="n"/>
-      <x:c r="D12" s="32" t="n"/>
-      <x:c r="E12" s="32" t="n"/>
-      <x:c r="F12" s="32" t="n"/>
-      <x:c r="G12" s="32" t="n"/>
-      <x:c r="H12" s="32" t="n"/>
-      <x:c r="I12" s="376" t="n"/>
-      <x:c r="J12" s="32" t="n"/>
-      <x:c r="K12" s="32" t="n"/>
-      <x:c r="L12" s="32" t="n"/>
-      <x:c r="M12" s="32" t="n"/>
+      <x:c r="A12" s="32" t="str">
+        <x:v>R-001</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="C12" s="32" t="str">
+        <x:v>Foundation</x:v>
+      </x:c>
+      <x:c r="D12" s="32" t="str">
+        <x:v>Platform monorepo bootstrap</x:v>
+      </x:c>
+      <x:c r="E12" s="32" t="str">
+        <x:v>Bootstrap the Section 74 skeleton and Stage 0 portable onboarding, verification, state, and handoff contract without implementing services or infrastructure.</x:v>
+      </x:c>
+      <x:c r="F12" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G12" s="32" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H12" s="32" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="I12" s="376" t="n">
+        <x:f>IF(H12="Done",1,IF(H12="In Progress",0.5,0))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J12" s="32" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="K12" s="32" t="str">
+        <x:v>Founder Stage 0</x:v>
+      </x:c>
+      <x:c r="L12" s="32" t="str">
+        <x:v>task verify: PASS; implementation commit 8a12c4489e078072bfef689c3bfbf5e8042b993c</x:v>
+      </x:c>
+      <x:c r="M12" s="32" t="str">
+        <x:v>Reconstructed with founder approval because R-001 through R-009 were absent from the supplied workbook.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" s="40" customFormat="1" ht="34" customHeight="1">
       <x:c r="A13" s="32" t="inlineStr">
@@ -21166,7 +21191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb9b5b7e13c748d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R308e65523c8a432d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): refresh commit evidence [R-001]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R53434dee85974d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R811d5e952e86496d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R1137bd330331448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R24fe666cb85f4a7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R25283bf47a754fcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rc91414faee36438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Re9ff0c04f09641c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Rc27ed19f114f430e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Re129f1cbb9904d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rbe55f94bbad54bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R5499cef0e3f34d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rdd1f17b2cb30447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R923b51ac0595453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Rf62e835aadc647d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rdf48a97b2ae148b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R7c58b57d949a4ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rd12114bcffd94601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rf6eb86bd258d4596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rb8ca52395bd34c29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R42dc08fe01ad4ad8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R2f791a86bea747a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R25f6899593e44230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R2627ba994766437a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R8209352158df40a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R8dd65bdd0cd84139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Raf1c3ff93da0451f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R0f40aef933c14f11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R90feb16396af48c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R551da609cef746cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R0fcc51ad90a5453a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rf7245d1c83844a9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rd1e09b7f635e48ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R6171d3d61e864a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R9530e900431c407e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R8445655acc534906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R0c7d5c727fc641b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Raa5c2c4fa6674e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R230e483b87e74047"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R1ff023cfe0924178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R13ebd64926b84e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R52389870c8024969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rffee81e084c34d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R19773a28afd04520"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R2862f88e3dc34d60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R5aa81de6bf5a4f5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R5693377c424a467f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R5f6c0f75bb9e4c29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rafb0645ceffe4d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rfc5b57c03fe240bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R9aeb6de9abdc4eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R0af15f49ea724801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rb938ba0233104cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rb2932757ae824c10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R2c590a6204d44fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Raae9fa6d54984c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R19798d42e55b4536"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R0c8b60a5550749d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rd0431f8af02b4055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R7f4f575efdca4c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rff01e373444f4e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rf404238e04de469c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R7dfd9445dc784c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcce5a4271fdd419c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R873991dd74de4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R2b4b18eb72474075"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Ree55d45e30354faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rd2cc8fce176d4fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rd7b95eb9440640e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R64f12543ff7c4d9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R5d6665c006d94d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R5841bf770ad4473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R391a0c040616469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Rca93e63580834734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R00d3a828e7dc42d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rec2790c465f14dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R6caab6076d9040f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R2ba545387a2e40f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R99e977f6e4d8475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R08bf5749087244a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Re01a644b94834c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Ra82be8d8d1ed4e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R5bb75f4bac5b45d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R7ffe4c646fe2492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R4cad4b62f2bb4760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R67c8cd945d9341ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R8613b7e33dea4624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Reffb609e029c4c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R486aa7ae100545a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R9557c25d386844ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R0f483e93beaa48bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Rdc731b3d155a401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Rb3c968e776c943ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rb1dada1a743a4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R405b08135a694214"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R893c054fd75a48af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R2f0052978a1d4240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Re328dc2fb7564d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R80b79a23ff0247e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rf7e068e013324921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R0960dad9b5214e24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rcf10b90fb6b84791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R4225c18de0134965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R0e2918abad244cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rf55fc6aa82e64253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R12186a36ce9045d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R690d1cba378444ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R5c94faac583d414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R45eaf74270a6410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R69ebcad7e3994a5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rbdd1d8e9f13c44b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rbbb70bf6e3a541a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rd223f13db0fb41fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rb302da5ddc5e4414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R9f49acb8c40c4fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rde2bcba4d86c497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R69a0cba04f0240dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Ra8c6771fcab04b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rda3adcc18fcf4e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rabf3efc9a1ff4d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rdbf6625df3dc4767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R96be7971c4124993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R3e1062837bed4356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rf85a4aca30c34e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R43213853d3fa49ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33dc2c58b3e24603"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1ee6919bce44265"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra941cc7dbd444fa7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe35812a2fe64fbb"/>
 </x:worksheet>
 </file>
 
@@ -10720,7 +10720,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L12" s="32" t="str">
-        <x:v>task verify: PASS; implementation commit 8a12c4489e078072bfef689c3bfbf5e8042b993c</x:v>
+        <x:v>task verify: PASS; implementation commit 655f01fa0425e8df9022ce6bb1d2040f56b1cb73</x:v>
       </x:c>
       <x:c r="M12" s="32" t="str">
         <x:v>Reconstructed with founder approval because R-001 through R-009 were absent from the supplied workbook.</x:v>
@@ -21191,7 +21191,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R308e65523c8a432d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138fe27d356948a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(data): bootstrap local postgres with pgvector [R-002]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcce5a4271fdd419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R873991dd74de4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R2b4b18eb72474075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Ree55d45e30354faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rd2cc8fce176d4fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rd7b95eb9440640e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R64f12543ff7c4d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R5d6665c006d94d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R5841bf770ad4473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R391a0c040616469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Rca93e63580834734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R00d3a828e7dc42d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rec2790c465f14dfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R6caab6076d9040f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R2ba545387a2e40f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R99e977f6e4d8475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R08bf5749087244a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Re01a644b94834c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Ra82be8d8d1ed4e01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R5bb75f4bac5b45d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R7ffe4c646fe2492c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R4cad4b62f2bb4760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R67c8cd945d9341ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R8613b7e33dea4624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Reffb609e029c4c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R486aa7ae100545a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R9557c25d386844ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R0f483e93beaa48bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Rdc731b3d155a401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Rb3c968e776c943ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rb1dada1a743a4e5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R405b08135a694214"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R893c054fd75a48af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R2f0052978a1d4240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Re328dc2fb7564d1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R80b79a23ff0247e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rf7e068e013324921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R0960dad9b5214e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rcf10b90fb6b84791"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R4225c18de0134965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R0e2918abad244cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rf55fc6aa82e64253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R12186a36ce9045d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R690d1cba378444ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R5c94faac583d414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R45eaf74270a6410c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R69ebcad7e3994a5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rbdd1d8e9f13c44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rbbb70bf6e3a541a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rd223f13db0fb41fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rb302da5ddc5e4414"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R9f49acb8c40c4fa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rde2bcba4d86c497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R69a0cba04f0240dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Ra8c6771fcab04b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rda3adcc18fcf4e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rabf3efc9a1ff4d67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rdbf6625df3dc4767"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R96be7971c4124993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R3e1062837bed4356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rf85a4aca30c34e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R43213853d3fa49ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R055dc900bf2241c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Ra031a499505a4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Racc121a9012349c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rf24acdf53d5640f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rc953ee98501742dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R23d0eac6df534487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R262c1aefed3346b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R7c39edeabce34a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rf7e4511bd0d34750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rae53df53fb2e4b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Rbe94df90b5aa4fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rcd4c8e4069fb4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rc421fbcf855c40bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R4b5d18a925ee44dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R6c51546179bb4080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R22b524276f274abd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R4ef8fa1b37534d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R2e813f8cde7b40d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R6e8830cb46154bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R000709e30b324215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R32ee06ef527748c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rb37354c0d353430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R997fa43272c74878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Rd1b0a06f73744779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Raffa046de9a74d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R34fd07f56a09401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="Rd4be4754cbf14140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Ra698f838b3c44a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R316da57ee7644c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R424e2f8462ae4378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Ref7493ba32574737"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R1b5b1b8ebe354f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rc845f6c0c26a4a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rdf97651bb4644c26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Rf3da740d1a5649a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R6002af1f50ac4998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R23e0bcb00b714400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Rf1bbcc12089c4400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R12b282c398c843ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R432209197d504cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rddaae48048f74a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rdeeb8b5438414bf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="Rd7e878b7f33c4506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rb3bf180fb85f4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R41d0fc2312a64676"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R32def2ff70a84778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rc2576c8541c94bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rff5b9ff7047041e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rd05cf17ea27e4644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6ec1e6f264814db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rb32cb386a2264d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R79d884b815464368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R6c08667853464a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R2269e45d1a884ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R37e001332890456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Re71c31b28a014bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Red3f4c4fc7e14e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R2892f2cde1cb4d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R828a973a1be34cf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R0cb5167682514729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R9f7ce3147da74f7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R8441a1c28a894bd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf1ee6919bce44265"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc435c82eb18c4027"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2702,7 +2702,7 @@
       </x:c>
       <x:c r="B5" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$B$4:$B$222,"MVP")</x:f>
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
@@ -2710,7 +2710,7 @@
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.009433962264150943</x:v>
+        <x:v>0.009345794392523364</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe35812a2fe64fbb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8b9323a55a45ff"/>
 </x:worksheet>
 </file>
 
@@ -10670,19 +10670,46 @@
       <x:c r="M10" s="32" t="n"/>
     </x:row>
     <x:row r="11" s="40" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A11" s="32" t="n"/>
-      <x:c r="B11" s="32" t="n"/>
-      <x:c r="C11" s="32" t="n"/>
-      <x:c r="D11" s="32" t="n"/>
-      <x:c r="E11" s="32" t="n"/>
-      <x:c r="F11" s="32" t="n"/>
-      <x:c r="G11" s="32" t="n"/>
-      <x:c r="H11" s="32" t="n"/>
-      <x:c r="I11" s="376" t="n"/>
-      <x:c r="J11" s="32" t="n"/>
-      <x:c r="K11" s="32" t="n"/>
-      <x:c r="L11" s="32" t="n"/>
-      <x:c r="M11" s="32" t="n"/>
+      <x:c r="A11" s="32" t="str">
+        <x:v>R-002</x:v>
+      </x:c>
+      <x:c r="B11" s="32" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="C11" s="32" t="str">
+        <x:v>Data</x:v>
+      </x:c>
+      <x:c r="D11" s="32" t="str">
+        <x:v>PostgreSQL + pgvector local bootstrap</x:v>
+      </x:c>
+      <x:c r="E11" s="32" t="str">
+        <x:v>Add local Docker Compose PostgreSQL with pgvector and a versioned initial migration.</x:v>
+      </x:c>
+      <x:c r="F11" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G11" s="32" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H11" s="32" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I11" s="376" t="n">
+        <x:f>IF(H11="Done",1,IF(H11="In Progress",0.5,0))</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J11" s="32" t="str">
+        <x:v>R-001</x:v>
+      </x:c>
+      <x:c r="K11" s="32" t="str">
+        <x:v>Founder Stage 0</x:v>
+      </x:c>
+      <x:c r="L11" s="32" t="str">
+        <x:v>task contract recorded; static Compose and migration checks pass</x:v>
+      </x:c>
+      <x:c r="M11" s="32" t="str">
+        <x:v>Reconstructed with founder approval from the kickoff kit's canonical R-002 example.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" s="40" customFormat="1" ht="34" customHeight="1">
       <x:c r="A12" s="32" t="str">
@@ -21191,7 +21218,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138fe27d356948a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedfc23c096340a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close local database bootstrap [R-002]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R055dc900bf2241c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Ra031a499505a4af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Racc121a9012349c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rf24acdf53d5640f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rc953ee98501742dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R23d0eac6df534487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R262c1aefed3346b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R7c39edeabce34a78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rf7e4511bd0d34750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rae53df53fb2e4b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Rbe94df90b5aa4fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rcd4c8e4069fb4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rc421fbcf855c40bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R4b5d18a925ee44dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R6c51546179bb4080"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R22b524276f274abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R4ef8fa1b37534d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R2e813f8cde7b40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R6e8830cb46154bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R000709e30b324215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R32ee06ef527748c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rb37354c0d353430f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R997fa43272c74878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Rd1b0a06f73744779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Raffa046de9a74d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R34fd07f56a09401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="Rd4be4754cbf14140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Ra698f838b3c44a41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R316da57ee7644c98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R424e2f8462ae4378"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Ref7493ba32574737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R1b5b1b8ebe354f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rc845f6c0c26a4a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rdf97651bb4644c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Rf3da740d1a5649a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R6002af1f50ac4998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R23e0bcb00b714400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Rf1bbcc12089c4400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R12b282c398c843ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R432209197d504cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rddaae48048f74a9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rdeeb8b5438414bf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="Rd7e878b7f33c4506"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rb3bf180fb85f4a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R41d0fc2312a64676"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R32def2ff70a84778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rc2576c8541c94bd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rff5b9ff7047041e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rd05cf17ea27e4644"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6ec1e6f264814db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rb32cb386a2264d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R79d884b815464368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R6c08667853464a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R2269e45d1a884ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R37e001332890456d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Re71c31b28a014bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Red3f4c4fc7e14e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R2892f2cde1cb4d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R828a973a1be34cf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R0cb5167682514729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R9f7ce3147da74f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R8441a1c28a894bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30dfdbe8a4214586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R6dd41cb6189e4b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rbf48f50fcaac4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Ra85df556ebf94f4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R7fc125ec1fcd4d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R689da3e4b9094b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R850485b156c84206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R4cc16544f20c4b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R4dc22b7c7c6444af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R62bf6f9031294e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Ra6f563bdafd44ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R5f10c292c36e4dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rc25e933c46374d0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R0828258b76844c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R0cf53487725d4b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R6f802ce7454b43eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rec6bf71fb99744d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R6895a9537831455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rbeb580ff773d400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R6fe18c14d8b64232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rcc6bb55f08a04baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rd41e25fa45eb4e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Rb963ed8edc634ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R08769eed11c44e29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rfb172b85f0b34f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Rfa4d88d47a504366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R18a1c0d254f94fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Rc29e70a6a9454333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R7aca78547cd84097"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R8608465f29334255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rbfcc86ad20d64ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R61ceca7a3a874a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R28a520315385444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R0244a1f44de34a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R254bde6a66284d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Ra798b0e058104f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rc73c81ef8cd047c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R81e1357580554d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rff75b2da3a7f4160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R4f2a7d62c167415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rdf96649e006c4689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Re1da4396c79e4c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R0ddbc8d377cc4023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R2976ceeb57ca4b6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="Rcf6d3a9f2a4f4b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="Rf78a8dbd791944d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R19641641136a4dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rac192eb5abaa4c52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rf905d382e27f4014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rb0247ad453a24341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R712f047b5b32411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Ra8f29b6cf15f4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R38dc9e50aac34516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Rdbea0b634cfd43e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R09317ba2a26c43cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Ra931e516b884493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Ra08ba73841a74cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R7ec8db2d04b74fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R7db43b5a5641498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R7fb527def27f4f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R79bdb25758404d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R4ba89d80aef74606"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc435c82eb18c4027"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e6d6ae1f3a04092"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2706,11 +2706,11 @@
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.009345794392523364</x:v>
+        <x:v>0.018691588785046728</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2803,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F8)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8b9323a55a45ff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1281b347a9d84fb2"/>
 </x:worksheet>
 </file>
 
@@ -10692,11 +10692,11 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H11" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I11" s="376" t="n">
         <x:f>IF(H11="Done",1,IF(H11="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="32" t="str">
         <x:v>R-001</x:v>
@@ -10705,7 +10705,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L11" s="32" t="str">
-        <x:v>task contract recorded; static Compose and migration checks pass</x:v>
+        <x:v>task verify: PASS; task db:verify: PostgreSQL healthy, pgvector 0.8.6, migration 1; implementation commit 56bf4b0dea5486f8d6dcde0c7b1054249ebbb064</x:v>
       </x:c>
       <x:c r="M11" s="32" t="str">
         <x:v>Reconstructed with founder approval from the kickoff kit's canonical R-002 example.</x:v>
@@ -21218,7 +21218,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcedfc23c096340a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R658fa812d75c4342"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(models): bootstrap local ollama runtime [R-003]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R30dfdbe8a4214586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R6dd41cb6189e4b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rbf48f50fcaac4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Ra85df556ebf94f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R7fc125ec1fcd4d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R689da3e4b9094b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R850485b156c84206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R4cc16544f20c4b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R4dc22b7c7c6444af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R62bf6f9031294e69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Ra6f563bdafd44ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R5f10c292c36e4dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rc25e933c46374d0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R0828258b76844c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R0cf53487725d4b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R6f802ce7454b43eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rec6bf71fb99744d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R6895a9537831455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rbeb580ff773d400f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R6fe18c14d8b64232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rcc6bb55f08a04baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rd41e25fa45eb4e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Rb963ed8edc634ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R08769eed11c44e29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rfb172b85f0b34f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Rfa4d88d47a504366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R18a1c0d254f94fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Rc29e70a6a9454333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R7aca78547cd84097"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R8608465f29334255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rbfcc86ad20d64ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R61ceca7a3a874a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R28a520315385444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R0244a1f44de34a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R254bde6a66284d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Ra798b0e058104f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rc73c81ef8cd047c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R81e1357580554d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rff75b2da3a7f4160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R4f2a7d62c167415e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rdf96649e006c4689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Re1da4396c79e4c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R0ddbc8d377cc4023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R2976ceeb57ca4b6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="Rcf6d3a9f2a4f4b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="Rf78a8dbd791944d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R19641641136a4dfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rac192eb5abaa4c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rf905d382e27f4014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rb0247ad453a24341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R712f047b5b32411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Ra8f29b6cf15f4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R38dc9e50aac34516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Rdbea0b634cfd43e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R09317ba2a26c43cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Ra931e516b884493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Ra08ba73841a74cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R7ec8db2d04b74fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R7db43b5a5641498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R7fb527def27f4f61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R79bdb25758404d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R4ba89d80aef74606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R00d7f0a73cdf45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Re0202e6fcad941e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R7b70692b89404357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rf4c6d44c25594c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rb342a0bf540748cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R7a737c0e45d34555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R24fe5548064d4c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R44e7375bbad245be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R78f01624e0e44a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rc3a7aab8c00b4532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R83a2a836b535473b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R2589996fc76d4b13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R2bc7c8c834664593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Ra9730933a1b846f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rd4403e296e024055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R472f54521621486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R8c22e830b0f348f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R04e83f3e37ae46bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R194b62c715e744af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R6e907ebfbed84f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rddd74835f85d4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R4d2d2429a2e74e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Radefe041470246a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Ra9c69dc89df84f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R95aa3bb8b3a743f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Rda1b821fc4dc4c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R04377a60c5d44424"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R37588fbc27304fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R44271d7c04d241aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R90b07ede2dca4ca0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R8b3343dbcff548b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rca8824d877014da0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rb1e066dadbc1470f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rd747f63dafe64618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R0c836f4f212c4dcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R36bd44e5fe17490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R3e86a50313c84742"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Re01fe66c50ab4c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rd50c265820004029"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R243381d39d8b43fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rb3ed12f7c3da4dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rf6c313ff76884794"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R5d94ba99ef304488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R62180abd8cfc4222"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R6b3544e4ab6e4f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R538e66e9adf24efd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R4e798b72d83b4704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R98b425bd4af24233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R3eb03668fe734ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6591e613a2cb4c56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Raa6db372f38142a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Ra402f6c81f584542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Ra05fc1aa689b49a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R96f7272ba3a24fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R69dd3172312a45fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R2d19f12323dd474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R7ce6120509624fe0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rd9a2385e5ffc4118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rfea6e29156754801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R1b60c1475e6846f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rfca6dd5e58d2488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R45af6a41d7104827"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3e6d6ae1f3a04092"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13cddeb11a084527"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2702,7 +2702,7 @@
       </x:c>
       <x:c r="B5" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$B$4:$B$222,"MVP")</x:f>
-        <x:v>107</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
@@ -2710,7 +2710,7 @@
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.018691588785046728</x:v>
+        <x:v>0.018518518518518517</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1281b347a9d84fb2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dae25eb44e74dc4"/>
 </x:worksheet>
 </file>
 
@@ -10655,19 +10655,46 @@
       <x:c r="M9" s="32" t="n"/>
     </x:row>
     <x:row r="10" s="40" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A10" s="32" t="n"/>
-      <x:c r="B10" s="32" t="n"/>
-      <x:c r="C10" s="32" t="n"/>
-      <x:c r="D10" s="32" t="n"/>
-      <x:c r="E10" s="32" t="n"/>
-      <x:c r="F10" s="32" t="n"/>
-      <x:c r="G10" s="32" t="n"/>
-      <x:c r="H10" s="32" t="n"/>
-      <x:c r="I10" s="376" t="n"/>
-      <x:c r="J10" s="32" t="n"/>
-      <x:c r="K10" s="32" t="n"/>
-      <x:c r="L10" s="32" t="n"/>
-      <x:c r="M10" s="32" t="n"/>
+      <x:c r="A10" s="32" t="str">
+        <x:v>R-003</x:v>
+      </x:c>
+      <x:c r="B10" s="32" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="C10" s="32" t="str">
+        <x:v>Models</x:v>
+      </x:c>
+      <x:c r="D10" s="32" t="str">
+        <x:v>Local Ollama Stage 0 bootstrap</x:v>
+      </x:c>
+      <x:c r="E10" s="32" t="str">
+        <x:v>Validate a loopback-only Ollama runtime, discover the configured local coder, and run a deterministic inference smoke test.</x:v>
+      </x:c>
+      <x:c r="F10" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G10" s="32" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H10" s="32" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I10" s="376" t="n">
+        <x:f>IF(H10="Done",1,IF(H10="In Progress",0.5,0))</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J10" s="32" t="str">
+        <x:v>R-002</x:v>
+      </x:c>
+      <x:c r="K10" s="32" t="str">
+        <x:v>Founder Stage 0</x:v>
+      </x:c>
+      <x:c r="L10" s="32" t="str">
+        <x:v>task contract recorded; existing local models discovered</x:v>
+      </x:c>
+      <x:c r="M10" s="32" t="str">
+        <x:v>Reconstructed with founder approval from Brief Sections 79 and 84.1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" s="40" customFormat="1" ht="34" customHeight="1">
       <x:c r="A11" s="32" t="str">
@@ -21218,7 +21245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R658fa812d75c4342"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e492d900a2a440d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close local ollama bootstrap [R-003]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R00d7f0a73cdf45ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Re0202e6fcad941e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R7b70692b89404357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rf4c6d44c25594c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rb342a0bf540748cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R7a737c0e45d34555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R24fe5548064d4c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R44e7375bbad245be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R78f01624e0e44a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rc3a7aab8c00b4532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R83a2a836b535473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R2589996fc76d4b13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R2bc7c8c834664593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Ra9730933a1b846f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rd4403e296e024055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R472f54521621486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R8c22e830b0f348f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R04e83f3e37ae46bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R194b62c715e744af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R6e907ebfbed84f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rddd74835f85d4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R4d2d2429a2e74e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Radefe041470246a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Ra9c69dc89df84f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R95aa3bb8b3a743f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Rda1b821fc4dc4c19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R04377a60c5d44424"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R37588fbc27304fbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R44271d7c04d241aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R90b07ede2dca4ca0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R8b3343dbcff548b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rca8824d877014da0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rb1e066dadbc1470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rd747f63dafe64618"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R0c836f4f212c4dcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R36bd44e5fe17490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R3e86a50313c84742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Re01fe66c50ab4c19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rd50c265820004029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R243381d39d8b43fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rb3ed12f7c3da4dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rf6c313ff76884794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R5d94ba99ef304488"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R62180abd8cfc4222"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R6b3544e4ab6e4f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R538e66e9adf24efd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R4e798b72d83b4704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R98b425bd4af24233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R3eb03668fe734ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6591e613a2cb4c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Raa6db372f38142a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Ra402f6c81f584542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Ra05fc1aa689b49a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R96f7272ba3a24fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R69dd3172312a45fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R2d19f12323dd474a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R7ce6120509624fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rd9a2385e5ffc4118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rfea6e29156754801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R1b60c1475e6846f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rfca6dd5e58d2488a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R45af6a41d7104827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Reb09c50866a4468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R7840e42548674cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R9069d6e5481849d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R3c542c3193b94325"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R2eb1dff453ed4a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R62e555690fc542be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Ra2d0c23a2f304d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R730012f6360a43a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Re7e6b3f16d2d440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R5377cc5b07324889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R9b8857cbb2334cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R0afa09499cd34be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R159eea6fa51e452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R30df471c68524bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Re70996f2e50c4645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R5d375f470d9b4d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rf1124f7814154b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R89a5f63759934c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Ra41f755ee044498f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R72d1f2dfdde94d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R270b5ffb660242f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rc2a1cb3189734183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R34979fe55fc74a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R42df6e56253e4b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rfe04e657137f43a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Re9d515345bf640bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R3f260f61bd5241ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R74a4fd70205442e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R899744d06c88468f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Rfc4ef13310d24b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R822e84e6b7cf4a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rbee77dbe4c7d4723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R5f85690d9665476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R4daaf45726794e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R6afe2279321740f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Rb052c1579dd848d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rccce0e7fe5f44386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Rbed796f6c7a34ad0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Re2e534ba97634b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R9e857ad26fc74191"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Re1dc9713f1f74161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R39ea44b2d3754a93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R7b45cb3435fd47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R8f33ac9219e94bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R18fd06a2f5f54a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R2d84666f629f424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rd154960bc7494c73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R7c4abb49f1e24ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R63b2009c5509487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R5046c29838cf4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R14a8ee372b0445fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R61b4c286f0d14e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rca8dccedfc6b47c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R12239c58f8004104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R49eaede7d7d04645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rb001f705c49e4437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R14553b24b76d4d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R811d3acb194841d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rce208b14e94b4831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R152813ae02224dd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rce52d7cf754742c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R20cfcd4158a54dc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13cddeb11a084527"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re23275222e1e45e8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2706,11 +2706,11 @@
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.018518518518518517</x:v>
+        <x:v>0.027777777777777776</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2803,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F8)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dae25eb44e74dc4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8872284e5de04766"/>
 </x:worksheet>
 </file>
 
@@ -10677,11 +10677,11 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H10" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I10" s="376" t="n">
         <x:f>IF(H10="Done",1,IF(H10="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="32" t="str">
         <x:v>R-002</x:v>
@@ -10690,7 +10690,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L10" s="32" t="str">
-        <x:v>task contract recorded; existing local models discovered</x:v>
+        <x:v>task verify: PASS; task ollama:verify: qwen2.5-coder:14b generated 6 tokens, cloud calls 0; implementation commit 822db27aa9c9e6ab836c28abba10f41dc27918d7</x:v>
       </x:c>
       <x:c r="M10" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 79 and 84.1.</x:v>
@@ -21245,7 +21245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e492d900a2a440d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b80298bf6640dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(control-plane): add stage 0 service foundation [R-004]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Reb09c50866a4468a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R7840e42548674cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R9069d6e5481849d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R3c542c3193b94325"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R2eb1dff453ed4a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R62e555690fc542be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Ra2d0c23a2f304d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R730012f6360a43a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Re7e6b3f16d2d440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R5377cc5b07324889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R9b8857cbb2334cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R0afa09499cd34be8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R159eea6fa51e452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R30df471c68524bed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Re70996f2e50c4645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R5d375f470d9b4d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rf1124f7814154b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R89a5f63759934c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Ra41f755ee044498f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R72d1f2dfdde94d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R270b5ffb660242f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rc2a1cb3189734183"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R34979fe55fc74a3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R42df6e56253e4b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rfe04e657137f43a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Re9d515345bf640bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R3f260f61bd5241ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R74a4fd70205442e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R899744d06c88468f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Rfc4ef13310d24b74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R822e84e6b7cf4a27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rbee77dbe4c7d4723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R5f85690d9665476c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R4daaf45726794e2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R6afe2279321740f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Rb052c1579dd848d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rccce0e7fe5f44386"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Rbed796f6c7a34ad0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Re2e534ba97634b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R9e857ad26fc74191"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Re1dc9713f1f74161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R39ea44b2d3754a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R7b45cb3435fd47d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R8f33ac9219e94bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R18fd06a2f5f54a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R2d84666f629f424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rd154960bc7494c73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R7c4abb49f1e24ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R63b2009c5509487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R5046c29838cf4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R14a8ee372b0445fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R61b4c286f0d14e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rca8dccedfc6b47c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R12239c58f8004104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R49eaede7d7d04645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rb001f705c49e4437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R14553b24b76d4d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R811d3acb194841d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rce208b14e94b4831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R152813ae02224dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rce52d7cf754742c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R20cfcd4158a54dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb4ccc713052b4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R540b9f24d02d40cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rcb178b95a2164083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R3de5e31164044f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R858ca87e1835447c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R0d4de921ce974731"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R651975375e484c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R490aff20e8aa456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R783299526cc64bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R71116ae298c34bdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R3ca67558595440c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R2c978254ba0f4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R09abb08cc8244bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Ra491fb970b734e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R0b8e92946a2049eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R34da357b6e344890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rab3cf2fd81454526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rc87f03b3cbf64bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rd42782c91d354a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="Rd53696d979fc4bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R87b2d2b1c5914afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R18d90eaead514ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R995bc5141b8c4503"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R81ce74a7a7344da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rb3d3a767a03b487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R39993b8f63014bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R15fbc9e1d9a5407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R9051549eb5824e0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R0960439038004bfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Re747810f50d844fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rfc6174ea7edd4440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R60d44a89af704a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rcd2c30fb3ac04584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rde1b59a000664582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R5af3faa1abe94c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R81bdff4576be4426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R9278920f2c514faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R41f12cfbd222427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R383388c0f16d4475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="Ra60a4641af924349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rae542ac6cc9843d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R93e4d227b1074e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="Rd1d7688c78714798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R6532fc594fcc4170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R98a7bdd6a6c94000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R31ed06484c784ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rdc8e807f31e54c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rb9603baae9274404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R9b3d7dbb6e3647fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rc2c31f286438446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R39ec5f09bae043a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rddc11a1a5ba14b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R5d323f184b8b46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Ra4882b061e3a45e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R622e70d707c44a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Re1f73e99dd084150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rb69ede4989964d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rbf159f1f0dda45cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R093045188c134686"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rb726a4e450a64ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R36dbced7b4554b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="Rfc5ddd21faea4623"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re23275222e1e45e8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R38439dbd57b74c0e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2702,7 +2702,7 @@
       </x:c>
       <x:c r="B5" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$B$4:$B$222,"MVP")</x:f>
-        <x:v>108</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
@@ -2710,7 +2710,7 @@
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.027777777777777776</x:v>
+        <x:v>0.027522935779816515</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8872284e5de04766"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbb6eb3f804405f"/>
 </x:worksheet>
 </file>
 
@@ -10640,19 +10640,46 @@
       </x:c>
     </x:row>
     <x:row r="9" s="40" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A9" s="32" t="n"/>
-      <x:c r="B9" s="32" t="n"/>
-      <x:c r="C9" s="32" t="n"/>
-      <x:c r="D9" s="32" t="n"/>
-      <x:c r="E9" s="32" t="n"/>
-      <x:c r="F9" s="32" t="n"/>
-      <x:c r="G9" s="32" t="n"/>
-      <x:c r="H9" s="32" t="n"/>
-      <x:c r="I9" s="376" t="n"/>
-      <x:c r="J9" s="32" t="n"/>
-      <x:c r="K9" s="32" t="n"/>
-      <x:c r="L9" s="32" t="n"/>
-      <x:c r="M9" s="32" t="n"/>
+      <x:c r="A9" s="32" t="str">
+        <x:v>R-004</x:v>
+      </x:c>
+      <x:c r="B9" s="32" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="C9" s="32" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="D9" s="32" t="str">
+        <x:v>Go control-plane foundation</x:v>
+      </x:c>
+      <x:c r="E9" s="32" t="str">
+        <x:v>Add the minimal Go modular-monolith service with typed configuration, liveness, PostgreSQL readiness, and graceful shutdown.</x:v>
+      </x:c>
+      <x:c r="F9" s="32" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G9" s="32" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H9" s="32" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="I9" s="376" t="n">
+        <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="J9" s="32" t="str">
+        <x:v>R-003</x:v>
+      </x:c>
+      <x:c r="K9" s="32" t="str">
+        <x:v>Founder Stage 0</x:v>
+      </x:c>
+      <x:c r="L9" s="32" t="str">
+        <x:v>local Ollama design review completed; implementation pending</x:v>
+      </x:c>
+      <x:c r="M9" s="32" t="str">
+        <x:v>Reconstructed with founder approval from Brief Sections 33, 74, and 84.1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" s="40" customFormat="1" ht="34" customHeight="1">
       <x:c r="A10" s="32" t="str">
@@ -21245,7 +21272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b80298bf6640dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4f620f4fdce4784"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close control-plane foundation [R-004]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb4ccc713052b4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R540b9f24d02d40cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rcb178b95a2164083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R3de5e31164044f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R858ca87e1835447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R0d4de921ce974731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R651975375e484c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R490aff20e8aa456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R783299526cc64bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R71116ae298c34bdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R3ca67558595440c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R2c978254ba0f4b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R09abb08cc8244bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Ra491fb970b734e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R0b8e92946a2049eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R34da357b6e344890"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rab3cf2fd81454526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rc87f03b3cbf64bb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rd42782c91d354a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="Rd53696d979fc4bb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R87b2d2b1c5914afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R18d90eaead514ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R995bc5141b8c4503"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R81ce74a7a7344da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rb3d3a767a03b487b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R39993b8f63014bde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R15fbc9e1d9a5407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R9051549eb5824e0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R0960439038004bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Re747810f50d844fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rfc6174ea7edd4440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R60d44a89af704a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rcd2c30fb3ac04584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rde1b59a000664582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R5af3faa1abe94c16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R81bdff4576be4426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R9278920f2c514faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R41f12cfbd222427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R383388c0f16d4475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="Ra60a4641af924349"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rae542ac6cc9843d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R93e4d227b1074e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="Rd1d7688c78714798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R6532fc594fcc4170"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R98a7bdd6a6c94000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R31ed06484c784ff2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rdc8e807f31e54c36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rb9603baae9274404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R9b3d7dbb6e3647fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rc2c31f286438446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R39ec5f09bae043a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rddc11a1a5ba14b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R5d323f184b8b46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Ra4882b061e3a45e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R622e70d707c44a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Re1f73e99dd084150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rb69ede4989964d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rbf159f1f0dda45cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R093045188c134686"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rb726a4e450a64ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R36dbced7b4554b9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="Rfc5ddd21faea4623"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc85171383c054e71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R612b52ccde644f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R4250bca6c9f743ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Reb2be2181f7d405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R586d117199014e54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Ra661b0fffea84c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R2abef9f7cdc74880"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R2361a2127f904c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rb5df949e707a4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R6ab5076f2b7e4577"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Re4d84e69d4ae4897"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rb94c9e7a22b94e3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R5582ca5198dc40ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="Ra1d66c352d2c4ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R652032e6c1d04b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="Rbae9157fb8884b81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R6580bfe76e3c49be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rb8b15d49279842ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rde93abb13fd14252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="Rd39641b674f94789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rb13320e7ff744ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R56f12e6076a3435c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Re8368796553d4247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R517910fcd8a244e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R983a36d0299a41fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Ra86dee9d2a9c4db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R7f08bc7885be46f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Ra71650951cec4ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Rf32cfc2b2eea4d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R7f8458654b194dbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R0d22e3d0a2f6473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rb2d3774d14cf4931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="Rdf2a80acbbba4a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Rf55d32b2b7c64f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R24aeae4dfd104fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R68c08163658941be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rf640f49bf9bc4a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R67835ae307b046a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rcec0af4665df49a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="Rac96ddb1c3d94a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R562d1b5a8efa441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R347a383d93314a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R01d6d3b14fc9480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R4c755ee167324704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R7fa5d0f607a84931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R894a58b01f394cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R1bebb3142e394bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rb5b3c5e13fa547cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Rc87df91e40724d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R7564129f8b4f4417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R097a31f299684ca0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R05025e72dbb04d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R4f95d019df3a4be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R3b68fb968a7f4d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Rbc097d41c0de4697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R1133ea33851e4337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rb7d7817ab6114cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rf5b1a44ab41e4322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rcf6192531f554001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rcc0c47f576bb4816"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rf2bdb7dea1ce47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R26b3945183de4664"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R38439dbd57b74c0e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6066a337ef949c7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2706,11 +2706,11 @@
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$222,"MVP",Phase_Roadmap!$H$4:$H$222,"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.027522935779816515</x:v>
+        <x:v>0.03669724770642202</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2803,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$222,F8)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbb6eb3f804405f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb869ef5424934a2d"/>
 </x:worksheet>
 </file>
 
@@ -10662,11 +10662,11 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-003</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>local Ollama design review completed; implementation pending</x:v>
+        <x:v>Implementation c44fd8d013e3ec1497ccb4ab55f1433df042aeb5; task verify, race tests, and live health/readiness passed; local_calls=1, cloud_calls=0</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 33, 74, and 84.1.</x:v>
@@ -21272,7 +21272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4f620f4fdce4784"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0812535af8224cf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close provider contract [R-005]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6fe0c7394c2c4173"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R9b457d3552314bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R015f6ec2e3c74bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rea1af2c3ec59434b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R7e40d7acfe784656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rcec0e5433a9a43ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R97993079f57c429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R0f6b282dc07f4a1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rdd8cd7e913504c21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Rc09b4f24f86945bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Rddd1a66f9c794d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R9738735dd5734ed9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Rd2edf97a36a943f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R768bc226d7374259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rf5bb56bdd83d4e0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R2cf1c7874db0410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Re57128e0544e432e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rd21cf4452f7b4753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R8ae30d5887754efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R12e6fdc17b6e4dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rf60ee456d0344472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R996bd6ff43cc4431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R733ec763525b480f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R27c2e4e333854918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R7d5528ead5af45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="Ra4db8b920d9c4be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R9a407171a56f4ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Ra7a6df0c03304818"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Rabb03fe1e98045be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R62ef2f30528b45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R5800f3eee6c94928"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R89a203449b404e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R8c7fd9786ca048b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R0fd40b2a82474d79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Re7ec11da982b421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Racb0941bda684ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R8071c4831e684dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Rcf1bc7ac9c344d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rb0974ce6637d4b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R22c5f79788a84fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R9fff97bc4e7842f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R78862bc09e724e17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R67c6f399987f49d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rf6092c8ff00c4ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="Rd7acda311c13443c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R683a50368b7c447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Re679b01840ad4f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Re0f5c2f114574f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R1ee02a1700d34c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R53c08a0f65434ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R1f6f19e685254a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R8a17b96582574383"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Rff43df5536974dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R8a565355e6914c3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Ra907ed9fc52a4b0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rbab94cf73e0e487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Ra7e5ebb528184871"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R6be7179bc7f54d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="Rc690be9ebbb7472d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R70fec2bf13a6481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Re6e6b83a921c452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R48be471dda0a46c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R845be9d295304bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R78f3e3fb4fae496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rac180c866b1e4178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R9e6c2e37dd5f4342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R7dea24a35661401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rb5aab34033b14156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Rd3789afc68334614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Rc06b768a4abd4183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rd37ccd6295e54869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R7a939b5a9aab4971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Ra9f689786cac4c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R27131bf574d44400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R4eab6978bb12416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R292eaa4bbb084c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R7d1342d4728c4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R85202e8c1b3545ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rf6f1735b9554478d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rcd6e018c51324fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rc514a667ea004f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R3ea8419881b74f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R7d4bd20a0b354f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="R88f40b52c2ec49c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R5135d552a9e24778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Rb73f4e4716584916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rb97a9680e13c4a6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R7b87c226d9734229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="Rdbe50d512a044841"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R2cd5303c50144c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="R45ffcdbb8103409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="Rd4ae7394511648e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R730be16c44794e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R010a0c65e87a4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R287fa46d3c274fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R42bbf45020c5475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R11e939439af8409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="Raa078d47216f46d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Re4b4d1c3d670450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R9bb01f58ef814582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R01e6340136484ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R1ef0bcd213bb40f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Ra769e92b63ea4306"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="R837b49f6b7d94d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R432535d648ce49f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rc9ba1133362748b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R75754a19c29b4b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R667dc0b877714b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Re524e032e9b24fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Racd97e2a22584194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R8dd7bec5c9e44c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="Rd954de2f302c440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R07b910a7caf04230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R4859bd9e08b0451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R122039b701d84cb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R8d94b2cc539c44ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R20342883c68f4bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R75dd23d8e20f4133"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rd0d8562bfeb74c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="Rc033f566ebc94e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R865d24e726f14025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R0835cc25f7e94356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R495180a7bd574d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="Rd074d9d6cb06487b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfe84f9b5d6194868"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R04b45655343f4593"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2706,11 +2706,11 @@
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$223,"MVP",Phase_Roadmap!$H$4:$H$223,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.03636363636363636</x:v>
+        <x:v>0.045454545454545456</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$223,F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2803,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$223,F8)</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7561346f29c413a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270cde4f50234b36"/>
 </x:worksheet>
 </file>
 
@@ -10662,11 +10662,11 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-004</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Task contract recorded; two local review attempts returned no capturable text; implementation pending; cloud_calls=0</x:v>
+        <x:v>Implementation afdc4ba9c14b231dece9533dbdd39e1e79e9ace3; task verify and 13 contract tests passed; local_calls=2 inconclusive, cloud_calls=0</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 18.3, 75, 83, 84, and 91.</x:v>
@@ -17998,7 +17998,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d0e3b741654a19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29fdf58ba6b6400d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close Ollama adapter [R-006]
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8f03f928e9ba40d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="Rb92228bb2ea645ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Re535e91e3cc34259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R822174bfda8745fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R2ac6ab7ab81b4289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R1ad22d7cf2f34458"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="Rfa6fde6cb7a145f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="R5df1b92fc1164dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R6aeab484d2e74963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R4aad5bc894b34909"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="Radec3e9ebc604ab2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R19d4c8ad021840c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Ra624480c3972480e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R4098bcc395dc405e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R21c1fc4892994710"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="Re1f0f06e306e4d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R7c391ea780614ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="Rf28ebb8ed52d4334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rd79a85621a8a4dab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R1f38e2b48a9a413e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rb1775eb2cec34d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Re518c3dc672c48a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="R69a3d106ec8e46ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="Raa6fab16bf9f4fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="Rc3a3a2877e5b40c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R4478a8d596dd4182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="Rb07c64ae7c6a4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Rbf3491ad6f584b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Ra8a68b8657ea4804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R5d29fd2913c94199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Re516337aabee4920"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R3a312b29ccd445e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R5b394eee0f5c449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R4ac34d5fa4f24ae4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="Rb3cb9f5d12b347bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R93cd1352d2dc4490"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Re46d1d63834b4f5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="Red5789bbba1a4ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="Rc0ddc73b071d44ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R0782e6079c7a478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R55cd8a9925994ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Rce8d44d0bad54f63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R58f1f2aebcdd4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R11f13a1b1233489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R5d4c79a934d042af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="Rc6e3d3915aa54d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Ra07966c5bdb14e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rcb3a6401d85d4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="R96afb7f00bb64d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R1218e8c40c8d406f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R59bcf14944f54e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R47c937dbff8248cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Raf27715a6ae349b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="Reb29ca4326794f5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="Rfad5282bea2b484c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R75e8c81fa61f4f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R82cf9543823848b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R96e00af2a7cf49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R7420459d16464482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rc9d477b006074375"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R5f6238433f4c46b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R57eae45e4b4c4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdd47f631d76f4f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R6659c2c1e684476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rade5cf8d8b8c40dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R47fcccdd55294144"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rf8da5ff482cc4570"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rf36c0fc8972b4284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R594a4884eff04ef1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Re8e7364a3dc6418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rbee1c0d403664a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R7b8fd3bf4f8e4bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R8a4be8acf5da489c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R676b5de3731c4b00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Ra7a7067d28594475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R87598fa7c6e64ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rc514f98e78b54a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="Re98f4d4cdb144b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rc1c9ae362a1a49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R2f31ab4a8b554852"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rd0da59769fe948a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R8d34430268224808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R5eeefb5b179942b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rb59729cc4aae4f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Rfc1d30cc496a45a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R58a6840c83394cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R66783a4fe9744e4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R17ffc502c10a483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R85a624b83eeb4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R97bc7939659947aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Ra3f48405b225477c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R85dfdb6f1c874061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rd61ad5399f3b459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R55e3ca6af5384808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R38946782d4c241a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R46d33a3983954ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R2cd8c72b11ba4411"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R20c487f1de5d4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R7fb0b2ed173a48c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R4a6ecba061314228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R5e44dd48774f43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R3dbfa3e7b92c4d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R8d8418c37f9b4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Re2cc9d491322436d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R05eb3f6114764ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rcbd0d9f7a92c4017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="Re36649bff8de4dfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R8f62d288f1304c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R510921099b754637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rd09153d947344a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Re2cb193628414591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6aaeb7f342b64683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rf7672bb4f89e4074"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rf828f2bc51d74e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Ra528ed05e55447c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R1883f721a0504c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R43bfe94ed6c34fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rf02ce2f567904d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rb8e4e43a80c14f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R3d1103fab0c74f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R9370d9fb8c90421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R9422248acb1f4058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R006ff08d348c4e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="Rce44d0fcf7c74d18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2379,7 +2379,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2d7e437deed84762"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6eca6997bd0b46f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2706,11 +2706,11 @@
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$224,"MVP",Phase_Roadmap!$H$4:$H$224,"Done")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.04504504504504504</x:v>
+        <x:v>0.05405405405405406</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2747,7 +2747,7 @@
       </x:c>
       <x:c r="G6" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$224,F6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2803,7 +2803,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$224,F8)</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3972,7 +3972,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dad15da017348e8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fb82ea71d4f4f7b"/>
 </x:worksheet>
 </file>
 
@@ -10662,11 +10662,11 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-005</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Task contract recorded; baseline task verify passed; local_calls=1 inconclusive, cloud_calls=0</x:v>
+        <x:v>Implementation 8061ca3b129539ada4b0838d7d70c8acd3df1ea3; task verify, adapter tests, and live loopback conformance passed; local_calls=3, cloud_calls=0</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 18.3, 75, 84, 85, 91, and 92.</x:v>
@@ -18040,7 +18040,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2f3baf1db734685"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d3181bed244ca5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close balanced model gateway router [R-007]
Mark R-007 done with verification evidence and record the completion state.

- task verify passed with 42 agent-engine tests (14 new gateway tests);
  security/env checks passed; Compose unchanged (postgres, control-plane).
- Routing is deterministic; zero local and zero cloud model calls.
- Tracker: R-007 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended by one row with no existing ID lost (MVP total 112, Done 7).
- Next: reconstruct R-008 (first cloud API-key adapter), pending an explicit
  founder decision on the paid provider.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-006</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-007-balanced-model-gateway; deterministic Balanced router and 14 offline gateway tests added; local_calls=0, cloud_calls=0.</x:v>
+        <x:v>Implementation 9faacd23dc22c6773f9a51dc58087d557c0be391; task verify passed with 42 agent-engine tests (14 new gateway tests); deterministic routing, local_calls=0, cloud_calls=0; Compose unchanged (postgres, control-plane).</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 18, 18.1, 18.2, 18.3, 84, 85, 91, and 92; founder intent to support both cloud API-key and local providers one at a time.</x:v>

</xml_diff>

<commit_message>
docs(state): close cloud provider adapters [R-008]
Mark R-008 done with verification evidence and record completion state.

- task verify passed with 61 agent-engine tests; security/env checks passed;
  Compose unchanged (postgres, control-plane); no cloud key set so cloud_calls=0.
- Tracker: R-008 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended by one row with no existing ID lost (MVP total 113, Done 8).
- Next: reconstruct R-009 (candidate true per-provider streaming or fallback).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-007</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-008-cloud-provider-adapters; multi-provider cloud adapters + env bootstrap + offline tests added; no cloud key set, cloud_calls=0.</x:v>
+        <x:v>Implementation eeade72e84c7f1ebd71dfc8c0f7c2f4db0f79677; task verify passed with 61 agent-engine tests (19 new cloud/bootstrap tests); no cloud key configured so cloud_calls=0; local gateway run works on qwen2.5-coder:14b and qwen3.5:9b; Compose unchanged (postgres, control-plane).</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (configure each provider; run locally on Ollama until keys are added) from Brief Sections 18, 18.3, 84, 85, 87, 90, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close usage and cost accounting [R-009]
Mark R-009 done with verification evidence and record completion state.

- task verify passed with 74 agent-engine tests; security/env checks passed;
  Compose unchanged; records are metadata-only; no model call to verify.
- Tracker: R-009 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended by one row with no existing ID lost (MVP total 114, Done 9).
- Next: reconstruct R-010 with founder confirmation (workbook R-010 is Native
  iOS Agent, which must wait for web/backend stability).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-008</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-009-usage-cost-accounting; usage/cost accounting records, price book, and ledger added; wired into the gateway; offline tests added; local_calls=0, cloud_calls=0.</x:v>
+        <x:v>Implementation f2fc8654c6a5717e292adcdc2abb5da2fd7409c2; task verify passed with 74 agent-engine tests (13 new accounting tests); deterministic accounting, metadata-only records, local_calls=0, cloud_calls=0; live gateway prints cost summary; Compose unchanged (postgres, control-plane).</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (best-in-class usage/cost accounting) from Brief Sections 18.4, 23, 68, 84, 85, 90, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close cloud SSE streaming [R-220]
Mark R-220 done with verification evidence and record completion state.

- task verify passed with 78 agent-engine tests; security/env pass; Compose
  unchanged; no cloud call (no key).
- Tracker: R-220 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended with no ID lost; backlog R-010 (Native iOS Agent) intact
  (MVP total 115, Done 10).
- Next: R-221 (confirmed second required item).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-009</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-220-cloud-streaming; true SSE streaming added for OpenAI-compatible, Anthropic, and Gemini adapters; offline parser tests added; cloud_calls=0.</x:v>
+        <x:v>Implementation 4e31841e730a6466da55843ff352f7144dd763e9; task verify passed with 78 agent-engine tests (5 new SSE streaming tests); true incremental streaming for OpenAI/Anthropic/Gemini; cloud_calls=0; Compose unchanged (postgres, control-plane).</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (complete both required items one by one) from Brief Sections 18, 57, 84, 85, 90, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close cross-provider fallback [R-221]
Mark R-221 done with verification evidence and record completion state.

- task verify passed with 86 agent-engine tests; security/env pass; Compose
  unchanged; single-provider behavior unchanged; no cloud call.
- Tracker: R-221 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended, no ID lost, backlog intact (MVP total 116, Done 11).
- Next: R-222 (first Next.js console slice).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-220</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-221-cross-provider-fallback; explicit fallback chain + per-provider circuit breaker added to the gateway; offline tests added; cloud_calls=0.</x:v>
+        <x:v>Implementation d0ee9f75b0d124fe60f1121b7f2a70d3b73040de; task verify passed with 86 agent-engine tests (8 new fallback/circuit-breaker tests); explicit allowlist fail-over + per-provider breaker; cloud_calls=0; Compose unchanged (postgres, control-plane).</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (complete both required items one by one) from Brief Sections 18, 18.3, 84, 89, 90, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close platform console slice [R-222]
Mark R-222 done with verification evidence and record completion state.

- task verify passed with 92 agent-engine tests; console served over HTTP
  (assets 200); no secret in snapshot; security/env pass; Compose unchanged.
- Tracker: R-222 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended, no ID lost, backlog intact (MVP total 117, Done 12).
- Next: confirm next Tracker ID (env-driven fallback wiring, or Next.js
  console upgrade once registry access is reliable).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-221</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-222-console-web; static platform console + Python overview exporter added; local_calls=0, cloud_calls=0.</x:v>
+        <x:v>Implementation c07bbcb1b9b8c010c6d64e3a0e09ac0c855102c8; task verify passed with 92 agent-engine tests (6 new overview tests); static console serves over HTTP (assets 200, 6 providers/5 prices/5 ladder), app.js node --check ok, no secret in snapshot; cloud_calls=0; Compose unchanged.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (advanced, smooth, secure platform) from Brief Sections 8, 15.2, 40, 41, 77, 90, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close env-driven fallback wiring [R-223]
Mark R-223 done with verification evidence and record completion state.

- task verify passed with 98 agent-engine tests; security/env pass; Compose
  and offline bootstrap unchanged; single-provider default unchanged.
- Tracker: R-223 recorded and marked Done at Phase_Roadmap row 9; ranges
  extended, no ID lost (MVP total 118, Done 13).
- Next: attempt R-224 (Next.js console upgrade), contingent on SWC install.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-221</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-223-env-fallback-wiring; env-driven fallback chain + circuit breaker + console resilience panel; cloud_calls=0.</x:v>
+        <x:v>Implementation 9ec809149ab91ebaa13b88ff0a15ebd382d7a728; task verify passed with 98 agent-engine tests (6 new); env-driven fallback chain + circuit breaker; default single-provider unchanged; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (complete remaining items one by one) from Brief Sections 18.3, 84, 87, 89, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close Application IR v1 [R-225]
Mark R-225 done with verification evidence and record completion state.

- task verify passed with 115 agent-engine tests (17 new IR tests); security/
  env pass; Compose and offline bootstrap unchanged.
- Tracker: R-225 (Product) recorded and marked Done at Phase_Roadmap row 9;
  ranges extended, no ID lost (MVP total 120, Done 14).
- Product roadmap recorded: R-226 adapter contract -> R-227 Next.js code
  adapter -> R-228 Git service -> (cloud env) sandbox/preview/deploy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-004</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-225-application-ir; validated versioned Application IR + tests; cloud_calls=0.</x:v>
+        <x:v>Implementation ad5e4ddf5918ddf3e4005c21a07c21601faf2ee6; task verify passed with 115 agent-engine tests (17 new IR tests); validated, versioned, framework-neutral Application IR with lossless serialization; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval to begin the actual product per Brief Sections 2, 9, 24, 47, 77, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close framework adapter contract [R-226]
Mark R-226 done with verification evidence and record completion state.

- task verify passed with 125 agent-engine tests (10 new codegen-contract
  tests); security/lint pass; Compose and offline bootstrap unchanged.
- Tracker: R-226 (Product) marked Done at Phase_Roadmap row 9; ranges extended,
  no ID lost (MVP total 121, Done 15).
- Next: R-227 Next.js web adapter (emit a real app from the IR).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-225</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-226-adapter-contract; codegen file-set + adapter contract + registry + tests.</x:v>
+        <x:v>Implementation f27bf416e99423d281e1c4e6f3eabc363848f95f; task verify passed with 125 agent-engine tests (10 new codegen-contract tests); pure in-memory file-set + adapter contract + registry; no disk writes; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 16, 17, 46, 47, 74, 75, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close Next.js web adapter [R-227]
Mark R-227 done with verification evidence and record completion state.

- task verify passed with 134 agent-engine tests (9 new); demo IR generates a
  13-file Next.js app; security/lint pass; Compose and offline bootstrap unchanged.
- Tracker: R-227 (Product) marked Done at Phase_Roadmap row 9; ranges extended,
  no ID lost (MVP total 122, Done 16).
- Next: R-228 Git service (materialize a GeneratedProject into a customer-owned
  repo + commit) — completes the first end-to-end builder slice.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-226</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-227-nextjs-adapter; Next.js web adapter emits a real app from the IR; tests.</x:v>
+        <x:v>Implementation 1a4f8a9b8cc2ca59be32142bb6c16992cb4dbd40; task verify passed with 134 agent-engine tests (9 new adapter/path tests); generates a 13-file Next.js app from the demo IR (entities-&gt;interfaces, {param}-&gt;[param] routes); no install/build/disk; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 9, 16, 40, 43, 46, 47, 74, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close git service — first builder slice complete [R-228]
Mark R-228 done with verification evidence and record completion state.

- task verify passed with 140 agent-engine tests (6 new git-service tests);
  security/lint pass; Compose and offline bootstrap unchanged.
- End-to-end demo: IR -> 13-file Next.js app -> one-commit customer-owned repo.
- Tracker: R-228 (Product) marked Done at Phase_Roadmap row 9; ranges extended,
  no ID lost (MVP total 123, Done 17).
- Milestone: first end-to-end builder slice (IR -> app -> owned repo) complete;
  next steps (sandbox/preview/deploy, backend adapter) need a cloud env.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-227</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on ai/R-228-git-service; materialize + repo init/commit + tests.</x:v>
+        <x:v>Implementation 28801ef396f7ead743a1d0cdc68657de23cefe1a; task verify passed with 140 agent-engine tests (6 new git-service tests); demo IR -&gt; 13-file Next.js app -&gt; one-commit customer-owned repo; writes only in target, no global git config, offline; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 6, 20, 34, 71, 74, 75, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close Python backend adapter; multi-target complete [R-229]
Mark R-229 done and record completion state. Session paused by founder.

- task verify passed with 147 agent-engine tests (7 new); one IR emits web
  (Next.js) + backend (FastAPI). Security/lint pass; Compose and offline
  bootstrap unchanged.
- Tracker: R-229 (Product) marked Done at Phase_Roadmap row 9 (MVP total 124,
  Done 18). Repo consolidated onto main (only branch; default).
- Next: R-230 Go backend adapter (offline), or sandbox/preview/deploy (cloud env).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-226</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on main; FastAPI backend adapter emits a backend from the IR; tests.</x:v>
+        <x:v>Implementation 04f1e6ad03ff52522efda81845ea3ee73e736a7d; task verify passed with 147 agent-engine tests (7 new); demo IR -&gt; 12-file Next.js web + 11-file FastAPI backend; no install/build/disk; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (multi-target from one IR) from Brief Sections 9, 16, 42, 43, 46, 47, 74, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close Go backend adapter; tri-target complete [R-230]
Mark R-230 done and record completion state.

- task verify passed with 154 agent-engine tests (7 new). One IR emits web
  (Next.js) + Python (FastAPI) + Go (net/http). Security/lint pass; Compose and
  offline bootstrap unchanged.
- Tracker: R-230 (Product) marked Done at Phase_Roadmap row 9 (MVP total 125,
  Done 19).
- Next: R-231 IR validator/normalizer + fixtures (offline), or
  sandbox/preview/deploy (cloud env).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-226</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>Implementation in progress on main; Go backend adapter emits a Go net/http service from the IR; tests.</x:v>
+        <x:v>Implementation e2515a8f1b0314ec287a02cdaf25e72a17b9da3f; task verify passed with 154 agent-engine tests (7 new); one IR -&gt; 12-file Next.js + 11-file FastAPI + 8-file Go service; no install/build/disk; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (multi-target from one IR) from Brief Sections 9, 16, 42, 43, 46, 47, 74, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close IR validator/normalizer + fixtures [R-231]
Mark R-231 done and record completion state.

- task verify passed with 163 agent-engine tests (9 new). Validator + canonical
  normalizer + example fixtures; construction checks unchanged. Security/lint
  pass; Compose and offline bootstrap unchanged.
- Tracker: R-231 (Product) marked Done at Phase_Roadmap row 9 (MVP total 126,
  Done 20).
- Near-term offline builder pieces complete; next steps (sandbox/preview/deploy,
  console upgrade) need a cloud/network environment.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-225</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress on main; IR validator/normalizer + example fixtures + tests.</x:v>
+        <x:v>Implementation f2027a6a7bc6bae37b14226838519c86657f8ff3; task verify passed with 163 agent-engine tests (9 new); validator + normalizer + 2 example fixtures; no dependency/network/model call; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 9, 12, 19, 66, 74, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close customer project assembler [R-232]
Mark R-232 done and record completion state.

- task verify passed with 169 agent-engine tests (6 new, incl. end-to-end
  materialize). One IR -> a 24-file customer monorepo -> an owned Git repo.
  Security/lint pass; Compose and offline bootstrap unchanged.
- Tracker: R-232 (Product) marked Done at Phase_Roadmap row 9 (MVP total 127,
  Done 21).
- The full OFFLINE builder is complete (spec -> IR -> adapters -> assembler ->
  Git repo). Next steps (sandbox/preview/deploy) need a cloud/network env.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-228</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress on main; customer project assembler + default registry + tests.</x:v>
+        <x:v>Implementation cf28cb0f46ae1f66b9f87b59232eceb2a113b508; task verify passed with 169 agent-engine tests (6 new); one IR -&gt; 24-file customer monorepo (apps/web + services/api) -&gt; owned Git repo in one commit; no install/build/disk; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval from Brief Sections 6, 34, 35, 46, 74, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close runtime & deploy provider layer [R-233]
Mark R-233 done and record completion state.

- task verify passed with 181 agent-engine tests (12 new). Local preview works
  (Tier 0/1); cloud sandbox/deploy providers activate by key (Tier 2/3).
  Security/lint/env pass; Compose and offline bootstrap unchanged; no key leak.
- Tracker: R-233 (Runtime) marked Done at Phase_Roadmap row 9 (MVP total 128,
  Done 22).
- Next: run a Tier-0 preview (network machine) or a concrete cloud driver once a
  key is provided.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-232</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress on main; runtime/deploy provider layer + local provider + env registry + tests.</x:v>
+        <x:v>Implementation ae11bac55fb9d865dbc6281c26f7df260edc3477; task verify passed with 181 agent-engine tests (12 new); local runtime works (Tier 0/1), cloud sandbox/deploy providers activate by key (Tier 2/3); no run/deploy, no secret leak; cloud_calls=0.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (wire Tier 0-3, keys plug in) from Brief Sections 15, 51, 55, 64, 75, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close tier switch + cloud provider drivers [R-234]
Tracker R-234 (Runtime) -> Done at impl dcb7d2d; MVP total 129, Done 23.
Records completion evidence (194 tests, verify/security/env pass, tier 0 and
tier 2 demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG,
CHANGELOG, and the resume prompt (built through R-234; continue from R-235).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-233</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done dcb7d2d — 194 tests (13 new); task verify + security:quick + env:check pass; platform:status demoed tier 0 and tier 2.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (one knob to switch tiers; all cloud providers get drivers) from Brief Sections 15, 51, 55, 64, 75, 91, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close verifiable-engineering verify plans [R-235]
Tracker R-235 (Verify) -> Done at impl cb74d0c; MVP total 130, Done 24.
Records completion evidence (203 tests, verify/security/env pass, verify-plan
demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
and the resume prompt (built through R-235; continue from R-236).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-232</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done cb74d0c — 203 tests (9 new); task verify + security:quick + env:check pass; verify-plan demoed for backend-go/nextjs-web; nothing installed/built/run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (verifiable engineering backbone) from Brief Sections 26, 27, 42, 44, 74, 77, 83, 84, 85, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close model-provider catalog expansion [R-236]
Tracker R-236 (Model Fabric) -> Done at impl e6326bf; MVP total 131, Done 25.
Records completion evidence (217 tests, verify/security/env pass, 12-provider
overview demoed incl. custom myco), refreshes PROJECT_STATE(.yaml/.md),
HANDOFF, WORK_LOG, CHANGELOG, and the resume prompt (built through R-236;
continue from R-237).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-223</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done e6326bf — 217 tests (14 new); task verify + security:quick + env:check pass; overview demoed 12-provider catalog incl. custom myco; no key value shown.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (add DeepSeek/Grok/etc. + custom/local providers, done the platform's way) from Brief Sections 10, 11, 12, 13, 55, 64, 69, 70, 74, 77, 90, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close IR-diff patch-apply edit loop [R-237]
Tracker R-237 (Builder) -> Done at impl a0a494a; MVP total 132, Done 26.
Records completion evidence (226 tests, verify/security/env pass, apply
round-trip + commit_edit history proven), refreshes PROJECT_STATE(.yaml/.md),
HANDOFF, WORK_LOG, CHANGELOG, and the resume prompt (built through R-237;
continue from R-238).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-232</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done a0a494a — 226 tests (9 new); task verify + security:quick + env:check pass; apply round-trip + commit_edit history proven; no network/exec, no write outside target.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (edit-an-app motion after generate + verify) from Brief Sections 6, 9, 27, 34, 35, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close PostgreSQL schema generation [R-238]
Tracker R-238 (Builder) -> Done at impl c6a4c6e; MVP total 133, Done 27.
Records completion evidence (237 tests, verify/security/env pass, schema +
FK demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
and the resume prompt (built through R-238; continue from R-239).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-232</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done c6a4c6e — 237 tests (11 new); task verify + security:quick + env:check pass; schema demoed for rideshare (driver + favourite_driver FK); no DB connection/run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (real persistence layer for the generated backend) from Brief Sections 9, 34, 35, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close data-access/repository layer [R-239]
Tracker R-239 (Builder) -> Done at impl f6792fa; MVP total 134, Done 28.
Records completion evidence (244 tests, verify/security/env pass, repos parse
+ Go struct scan), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG,
CHANGELOG, PROGRESS (MVP 20.9%, overall 11.7%), and the resume prompt
(built through R-239; continue from R-240).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-238</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done f6792fa — 244 tests (7 new); task verify + security:quick + env:check pass; python repos parse + go store scans model structs; parameterized SQL; no DB connection.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (make the generated backend use the schema) from Brief Sections 9, 34, 35, 42, 74, 77, 90, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close route wiring [R-240]
Tracker R-240 (Builder) -> Done at impl 013dfc4; MVP total 135, Done 29.
Records completion evidence (256 tests, verify/security/env pass, wired
routers/handlers demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF,
WORK_LOG, CHANGELOG, PROGRESS, and the resume prompt (built through R-240;
continue from R-241).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-239</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 013dfc4 — 256 tests (12 new); task verify + security:quick + env:check pass; Python routers call repositories, Go main opens store.Open()+handlers.New(db); ambiguous routes stay 501; nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (turn the 501 stubs into real CRUD over the data-access layer) from Brief Sections 9, 27, 34, 35, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close authentication guards [R-241]
Tracker R-241 (Builder) -> Done at impl 4db716b; MVP total 136, Done 30.
Records completion evidence (265 tests, verify/security/env pass, auth guards
demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
PROGRESS, and the resume prompt (built through R-241; continue from R-242).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-240</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 4db716b — 265 tests (9 new); task verify + security:quick + env:check pass; auth=true routes guarded (Python Depends, Go RequireAuth), public routes untouched; token verification is a documented TODO.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (enforce the IR auth flag; a core real-app feature) from Brief Sections 9, 27, 34, 35, 55, 64, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close real JWT verification [R-242]
Tracker R-242 (Builder) -> Done at impl e0d8af3; MVP total 137, Done 31.
Records completion evidence (268 tests, verify/security/env pass, JWT guards
demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
PROGRESS, and the resume prompt (built through R-242; continue from R-243).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-241</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done e0d8af3 — 268 tests (3 new); task verify + security:quick + env:check pass; Python require_auth uses PyJWT HS256, Go RequireAuth uses golang-jwt; JWT_SECRET from env only; nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (real token verification after the R-241 auth guard) from Brief Sections 9, 27, 34, 55, 64, 74, 77, 90, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close per-endpoint role enforcement [R-243]
Tracker R-243 (Builder) -> Done at impl 1faea2c; MVP total 138, Done 32.
Records completion evidence (274 tests, verify/security/env pass, role guards
demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
PROGRESS, and the resume prompt (built through R-243; continue from R-244).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-242</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 1faea2c — 274 tests (6 new); task verify + security:quick + env:check pass; IR required_roles validated+serialized, Python require_roles + Go RequireRoles -&gt; 403; validate_ir errors on unknown role; nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (per-endpoint roles after JWT verification) from Brief Sections 9, 27, 34, 55, 64, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close sub-collection route wiring [R-244]
Tracker R-244 (Builder) -> Done at impl b886d72; MVP total 139, Done 33.
Records completion evidence (285 tests, verify/security/env pass, sub-collection
lists demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
PROGRESS, and the resume prompt (built through R-244; continue from R-245).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-243</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done b886d72 — 285 tests (11 new); task verify + security:quick + env:check pass; GET /posts/{postId}/comments wired to list_comment_by_post (Py) / ListCommentByPost (Go); ambiguous routes stay 501; nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (finish the CRUD story via sub-collection lists) from Brief Sections 9, 27, 34, 35, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close combined project-plan surface [R-245]
Tracker R-245 (Runtime) -> Done at impl 891144d; MVP total 140, Done 34.
Records completion evidence (291 tests, verify/security/env pass, plan:show
demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG,
PROGRESS, and the resume prompt (built through R-245; continue from R-246).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10662,11 +10662,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-235</x:v>
@@ -10675,7 +10675,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 891144d — 291 tests (6 new); task verify + security:quick + env:check pass; task plan:show renders preview+verify per app; deploy opt-in; JSON secret-free; nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (one plan surface tying runtime + verify + deploy) from Brief Sections 15, 26, 27, 51, 74, 75, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close hunk-level edit diffs [R-246]
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -2,68 +2,68 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rdd47f631d76f4f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R6659c2c1e684476c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="Rade5cf8d8b8c40dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="R47fcccdd55294144"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="Rf8da5ff482cc4570"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="Rf36c0fc8972b4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R594a4884eff04ef1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Re8e7364a3dc6418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="Rbee1c0d403664a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="R7b8fd3bf4f8e4bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R8a4be8acf5da489c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="R676b5de3731c4b00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="Ra7a7067d28594475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R87598fa7c6e64ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rc514f98e78b54a12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="Re98f4d4cdb144b95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="Rc1c9ae362a1a49b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R2f31ab4a8b554852"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="Rd0da59769fe948a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="R8d34430268224808"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="R5eeefb5b179942b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rb59729cc4aae4f8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Rfc1d30cc496a45a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R58a6840c83394cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R66783a4fe9744e4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R17ffc502c10a483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R85a624b83eeb4526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="R97bc7939659947aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Ra3f48405b225477c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R85dfdb6f1c874061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="Rd61ad5399f3b459e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="R55e3ca6af5384808"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R38946782d4c241a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="R46d33a3983954ded"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R2cd8c72b11ba4411"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R20c487f1de5d4250"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="R7fb0b2ed173a48c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R4a6ecba061314228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R5e44dd48774f43f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R3dbfa3e7b92c4d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="R8d8418c37f9b4cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Re2cc9d491322436d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R05eb3f6114764ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="Rcbd0d9f7a92c4017"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="Re36649bff8de4dfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R8f62d288f1304c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="R510921099b754637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="Rd09153d947344a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Re2cb193628414591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R6aaeb7f342b64683"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="Rf7672bb4f89e4074"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="Rf828f2bc51d74e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="Ra528ed05e55447c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R1883f721a0504c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R43bfe94ed6c34fe3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="Rf02ce2f567904d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="Rb8e4e43a80c14f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R3d1103fab0c74f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R9370d9fb8c90421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="R9422248acb1f4058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="R006ff08d348c4e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="Rce44d0fcf7c74d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6da10e156e2345f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase_Roadmap" sheetId="2" r:id="R710097a944b547a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_UI_Tabs" sheetId="3" r:id="R0612ee88b50e4f17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Architecture" sheetId="4" r:id="Rf03bcca19e944f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Application_IR" sheetId="5" r:id="R098f665b79fe4be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_Impact" sheetId="6" r:id="R145229c062d94cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Build_Matrix" sheetId="7" r:id="R5f4c3caf817a4ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing_Quality" sheetId="8" r:id="Rc1207259f4754464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="9" r:id="R7b77d91700eb4858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Infrastructure" sheetId="10" r:id="Ra4f85646da2d4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Costs" sheetId="11" r:id="R313e3c20bdcd4153"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics_KPIs" sheetId="12" r:id="Rf51a36618d364463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks_Competitor" sheetId="13" r:id="R3dbf9c54a7ae4a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Gates" sheetId="14" r:id="R51a31206d142410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R26e2c03aa5dd4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Selection" sheetId="16" r:id="R1d75031f42a14f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework_Decision" sheetId="17" r:id="R0230f4a8764f45fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repo_Architecture" sheetId="18" r:id="R8d1d0156584145f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Structure" sheetId="19" r:id="R7e0967e91b054538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack_Profiles" sheetId="20" r:id="Rc6aadd8c4f8f4f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Sharing" sheetId="21" r:id="Rad59f5c2c00e4dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Architecture" sheetId="22" r:id="Rf1d634969dff4591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git_Standards" sheetId="23" r:id="Rac0b47daf8f1407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flutter_Template" sheetId="24" r:id="R2ec14c3ab2e44e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReactNative_Template" sheetId="25" r:id="R7a3065d20606479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Android_Template" sheetId="26" r:id="R90490284a9ff438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iOS_Template" sheetId="27" r:id="R89e84136129845f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web_Template" sheetId="28" r:id="Rfeb689b930f04818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin_Template" sheetId="29" r:id="Rf4766c8d86954963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Templates" sheetId="30" r:id="R7b00223709104ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_CD" sheetId="31" r:id="R98370e92bb2b4b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Paths" sheetId="32" r:id="Rbe691e9e28644c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template_Governance" sheetId="33" r:id="R4f2b4eed7e844772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference_Study" sheetId="34" r:id="Re38c260465904510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime_Tiers" sheetId="35" r:id="R3e5502f5845242b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Durable_Agent_Runtime" sheetId="36" r:id="R4b03cbcfc49840ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCP_Tool_Registry" sheetId="37" r:id="Rd3d64a032a724360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HITL_Approvals" sheetId="38" r:id="R421221b1f5a54f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution_Modes" sheetId="39" r:id="R66b76d025d724ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend_Profiles" sheetId="40" r:id="R863ca79915f248fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent_Streaming" sheetId="41" r:id="Rb4259bc3ad2043dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture_Research" sheetId="42" r:id="Ra3c3b33b066d45bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team_Glossary" sheetId="43" r:id="R3ee3a16c55054402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand_Naming" sheetId="44" r:id="R61627e393e6748ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview_Verification" sheetId="45" r:id="R10f72cf5f3df4fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Device_QR_Delivery" sheetId="46" r:id="R3683da26361f49df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Context_Engine" sheetId="47" r:id="Rc118420f830e4ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Memory" sheetId="48" r:id="R7e3f02617737489f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LLM_Cost_Optimization" sheetId="49" r:id="Re2ddde72a24e40a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Database_Strategy" sheetId="50" r:id="R3632d0d79f9c436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident_Bug_Flow" sheetId="51" r:id="R7916d36c67644b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor_Matrix" sheetId="52" r:id="R4992038a0c784d3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client_Handover" sheetId="53" r:id="R53a17e40ab714bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publishing_Release" sheetId="54" r:id="R5f342ca7743e40b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit_Economics" sheetId="55" r:id="R88658c78261649bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider_Interfaces" sheetId="56" r:id="R3cfa1c6ee33f435c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply_Chain" sheetId="57" r:id="R8097555c54f94ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RND_Gap_Audit" sheetId="58" r:id="R16011c52f79a4182"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Local_LLM_Providers" sheetId="59" r:id="R4ab85df1ed744db5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Developer_Handoff" sheetId="60" r:id="Rdaa2e8ae5c1f4cc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment_Matrix" sheetId="61" r:id="Rc8a3d54de32a4db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model_Capability_Registry" sheetId="62" r:id="R642d664b80a241c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1795,7 +1795,35 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="48">
+  <x:dxfs count="52">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEAF2F8"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF3F4F6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -2379,7 +2407,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6eca6997bd0b46f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a2adc8f129a4b86"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2389,21 +2417,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoadmapTable" displayName="RoadmapTable" ref="A3:M143" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoadmapTable" displayName="RoadmapTable" ref="A4:M254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
-    <x:tableColumn id="1" name="ID"/>
-    <x:tableColumn id="2" name="Phase"/>
-    <x:tableColumn id="3" name="Area"/>
-    <x:tableColumn id="4" name="Requirement"/>
-    <x:tableColumn id="5" name="Simple Description"/>
-    <x:tableColumn id="6" name="Priority"/>
-    <x:tableColumn id="7" name="Owner"/>
-    <x:tableColumn id="8" name="Status"/>
-    <x:tableColumn id="9" name="Completion %"/>
-    <x:tableColumn id="10" name="Dependency"/>
-    <x:tableColumn id="11" name="Target Sprint"/>
-    <x:tableColumn id="12" name="Evidence / Link"/>
-    <x:tableColumn id="13" name="Notes"/>
+    <x:tableColumn id="1" name="Phase"/>
+    <x:tableColumn id="2" name="Primary Outcome"/>
+    <x:tableColumn id="3" name="Mobile"/>
+    <x:tableColumn id="4" name="Web/Admin"/>
+    <x:tableColumn id="5" name="Backend/DB"/>
+    <x:tableColumn id="6" name="Context/Memory"/>
+    <x:tableColumn id="7" name="Runtime/Preview"/>
+    <x:tableColumn id="8" name="Workflow/Agents"/>
+    <x:tableColumn id="9" name="Git/Delivery"/>
+    <x:tableColumn id="10" name="Security"/>
+    <x:tableColumn id="11" name="Cost Focus"/>
+    <x:tableColumn id="12" name="Enterprise"/>
+    <x:tableColumn id="13" name="Gate"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2702,15 +2730,15 @@
       </x:c>
       <x:c r="B5" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$B$4:$B$254,"MVP")</x:f>
-        <x:v>111</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C5" s="32" t="n">
         <x:f>COUNTIFS(Phase_Roadmap!$B$4:$B$254,"MVP",Phase_Roadmap!$H$4:$H$254,"Done")</x:f>
-        <x:v>6</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D5" s="376" t="n">
         <x:f>IF(B5=0,0,C5/B5)</x:f>
-        <x:v>0.05405405405405406</x:v>
+        <x:v>0.24822695035460993</x:v>
       </x:c>
       <x:c r="F5" s="32" t="inlineStr">
         <x:is>
@@ -2803,7 +2831,7 @@
       </x:c>
       <x:c r="G8" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$254,F8)</x:f>
-        <x:v>6</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2814,7 +2842,7 @@
       </x:c>
       <x:c r="G9" s="32" t="n">
         <x:f>COUNTIF(Phase_Roadmap!$H$4:$H$254,F9)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10"/>
@@ -3972,7 +4000,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fb82ea71d4f4f7b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd09cf3b0f3d4893"/>
 </x:worksheet>
 </file>
 
@@ -10662,11 +10690,11 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
         <x:f>IF(H9="Done",1,IF(H9="In Progress",0.5,0))</x:f>
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-237</x:v>
@@ -10675,7 +10703,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done eebab68 — 297 tests (6 new); task verify + security:quick + env:check pass; diff_report gives hunk diffs + rename detection; unified_patch byte-stable; additive, nothing run.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (edits read as focused patches) from Brief Sections 6, 9, 27, 34, 74, 77, and 92.</x:v>
@@ -19266,7 +19294,21 @@
       <x:formula>H4="Deferred"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="10">
+  <x:conditionalFormatting sqref="H4:H254">
+    <x:cfRule type="expression" dxfId="48" priority="5">
+      <x:formula>H4="Done"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="49" priority="6">
+      <x:formula>H4="In Progress"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="50" priority="7">
+      <x:formula>H4="Blocked"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="51" priority="8">
+      <x:formula>H4="Deferred"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="13">
     <x:dataValidation type="list" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="B4:B143">
       <x:formula1>"MVP,MID,ADVANCED,PRODUCTION"</x:formula1>
     </x:dataValidation>
@@ -19297,10 +19339,19 @@
     <x:dataValidation type="list" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="F4:F252">
       <x:formula1>"P0,P1,P2,P3"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B4:B254">
+      <x:formula1>"MVP,MID,ADVANCED,PRODUCTION"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F4:F254">
+      <x:formula1>"P0,P1,P2,P3"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H4:H254">
+      <x:formula1>"Not Started,In Progress,Blocked,Done,Deferred"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d3181bed244ca5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f0d79c3295a447a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(state): close IR fixtures + seed migration [R-248]
Tracker R-248 (Builder) -> Done at impl 9d34720; MVP total 142, Done 37.
Records completion evidence (316 tests, verify/security/env pass, seed demoed),
refreshes PROJECT_STATE(.yaml/.md), HANDOFF, WORK_LOG, CHANGELOG, PROGRESS, and
the resume prompt (built through R-248; continue from R-249).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10718,10 +10718,10 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-247</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 9d34720 — 316 tests (14 new); task verify + security:quick + env:check pass; render_postgres_seed emits authored INSERTs (quoted/escaped), both backends emit 0002_seed.sql for minimal-blog, none for fixture-free/non-postgres; no DB connection, no fabricated value.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (honest seed data from explicit IR fixtures) from Brief Sections 9, 26, 27, 34, 35, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close schema indexes + unique constraints [R-249]
Tracker R-249 (Builder) -> Done at impl 28e7cd5; MVP total 143, Done 38.
Records completion evidence (327 tests, verify/security/env pass, unique +
index rendering demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF,
WORK_LOG, CHANGELOG, PROGRESS, and the resume prompt (built through R-249;
continue from R-250).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10718,10 +10718,10 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-248</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 28e7cd5 — 327 tests (11 new); task verify + security:quick + env:check pass; UNIQUE columns + CREATE [UNIQUE] INDEX rendered, id never unique, bad index field is a construction error, IR round-trips; no DB connection.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (deeper IR/adapter coverage: indexes + unique constraints) from Brief Sections 9, 34, 35, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close field validation into schema + models [R-250]
Tracker R-250 (Builder) -> Done at impl 1eed171; MVP total 144, Done 39.
Records completion evidence (337 tests, verify/security/env pass, VARCHAR/CHECK
+ Field/Literal demoed), refreshes PROJECT_STATE(.yaml/.md), HANDOFF,
WORK_LOG, CHANGELOG, PROGRESS, and the resume prompt (built through R-250;
continue from R-251).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10718,10 +10718,10 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-249</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 1eed171 — 337 tests (10 new); task verify + security:quick + env:check pass; STRING max_length -&gt; VARCHAR(n), enum -&gt; CHECK, Pydantic Field(max_length)/Literal; unknown rules ignored; examples unchanged; no DB connection.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (richer field validation into models + schema) from Brief Sections 9, 26, 27, 34, 42, 74, 77, and 92.</x:v>

</xml_diff>

<commit_message>
docs(state): close field validation for Go + numeric min/max [R-251]
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
+++ b/R_&_D/OmniStackAI_Execution_Tracker_v6.xlsx
@@ -10718,10 +10718,10 @@
         <x:v>Claude (Opus 4.8)</x:v>
       </x:c>
       <x:c r="H9" s="32" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I9" s="376" t="n">
-        <x:v>0.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="32" t="str">
         <x:v>R-250</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>Founder Stage 0</x:v>
       </x:c>
       <x:c r="L9" s="32" t="str">
-        <x:v>In progress — impl commit pending.</x:v>
+        <x:v>Done 2060a21 — 345 tests (8 new); task verify + security:quick + env:check pass; numeric CHECK + Pydantic ge/le + Go validate tags across all targets; rule-free fields unchanged; no go.mod dep, no DB connection.</x:v>
       </x:c>
       <x:c r="M9" s="32" t="str">
         <x:v>Reconstructed with founder approval (extend field validation to Go + numeric bounds) from Brief Sections 9, 26, 27, 34, 42, 74, 77, and 92.</x:v>

</xml_diff>